<commit_message>
Remove site-specific identifiers from the SLURM profiles
The three profiles hardcoded --mail-user=ppssingh@ucdavis.edu, so anyone
running this pipeline would have mailed their job notifications to its author.
Notifications are now commented out with an example to fill in.

slurm_account/partition/qos are UC Davis FARM values and are now labelled as
site-specific, since the scheduler at another site will reject them.

The intake workbook's email example is now a neutral placeholder.
</commit_message>
<xml_diff>
--- a/intake_template.xlsx
+++ b/intake_template.xlsx
@@ -810,7 +810,7 @@
       <c r="C6" s="10" t="inlineStr"/>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Where SLURM job notifications go. Example: yourname@ucdavis.edu</t>
+          <t>Where SLURM job notifications go. Example: you@example.edu</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       <c r="C6" s="10" t="inlineStr"/>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Where SLURM job notifications go. Example: yourname@ucdavis.edu</t>
+          <t>Where SLURM job notifications go. Example: you@example.edu</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       <c r="C6" s="10" t="inlineStr"/>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Where SLURM job notifications go. Example: yourname@ucdavis.edu</t>
+          <t>Where SLURM job notifications go. Example: you@example.edu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: expose bulk methods and reference controls in intake schema 4
</commit_message>
<xml_diff>
--- a/intake_template.xlsx
+++ b/intake_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re2ab5c6d1a9c426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk RNA-seq" sheetId="2" r:id="R2e7c11f3cabd4af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAGseq" sheetId="3" r:id="R1c7e1463cb6f45a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sRNA-seq" sheetId="4" r:id="Rd75b59d1e68a4cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samples" sheetId="5" r:id="Ra74a2a8ba39d4008"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Libraries" sheetId="6" r:id="Rafa898603ad7442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reads" sheetId="7" r:id="Re4976f2dea80472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R52182935ba874c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk RNA-seq" sheetId="2" r:id="Rcd36cd2ef9934461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAGseq" sheetId="3" r:id="R02685295f5d746c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sRNA-seq" sheetId="4" r:id="Rc85db9ae5f5744a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samples" sheetId="5" r:id="R06a01f7a5a3140ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Libraries" sheetId="6" r:id="R67d8b9055e90469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reads" sheetId="7" r:id="R0a54bcb5d2d44fc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -106,8 +106,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -164,6 +169,11 @@
         <x:fgColor rgb="FF2E7D32"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F5F5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -185,7 +195,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="63">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -357,6 +367,25 @@
     <x:xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="15" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="15" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -661,7 +690,7 @@
         <x:v>Template schema version</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -674,7 +703,7 @@
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="48" t="str">
-        <x:v>Current execution: annotated, non-UMI bulk gene expression and differential expression; independent groups, optionally including a batch column.</x:v>
+        <x:v>Current execution: annotated, non-UMI bulk gene expression and differential expression; Salmon or STAR, explicit fixed-effect methods, independent groups with optional batch.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
@@ -739,12 +768,12 @@
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="48" t="str">
-        <x:v>The current model compares all levels of the primary factor. Advanced contrasts, subject effects, reference overrides and execution settings still require configuration outside this workbook.</x:v>
+        <x:v>Bulk method, custom references and basic preprocessing have input fields. Advanced contrasts, subject effects, analysis objectives and executor settings still require configuration outside this workbook.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="48" t="str">
-        <x:v>Blank strandedness knowledge is not a reverse-stranded assumption: choose don't know. Salmon detects library type and reports disagreement with declared expectations.</x:v>
+        <x:v>Blank strandedness knowledge is not a reverse-stranded assumption: choose don't know. Salmon detects library type and reports disagreement. STAR requires a known declared strand; it does not infer strand.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -1235,12 +1264,172 @@
         <x:v>library_kit</x:v>
       </x:c>
     </x:row>
+    <x:row r="30" ht="51" customHeight="1">
+      <x:c r="A30" s="66" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B30" s="66" t="str">
+        <x:v>Bulk quantification method</x:v>
+      </x:c>
+      <x:c r="C30" s="68" t="str">
+        <x:v>auto</x:v>
+      </x:c>
+      <x:c r="D30" s="20" t="str">
+        <x:v>auto selects Salmon for gene expression. STAR needs a compatible genome/GTF and known strand.</x:v>
+      </x:c>
+      <x:c r="E30" s="39" t="str">
+        <x:v>analysis_quantifier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="51" customHeight="1">
+      <x:c r="A31" s="66" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="66" t="str">
+        <x:v>Differential expression method</x:v>
+      </x:c>
+      <x:c r="C31" s="68" t="str">
+        <x:v>auto</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>auto selects limma-voom for this independent design. Explicit methods keep the declared model.</x:v>
+      </x:c>
+      <x:c r="E31" s="39" t="str">
+        <x:v>analysis_backend</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="51" customHeight="1">
+      <x:c r="A32" s="66" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B32" s="66" t="str">
+        <x:v>Custom genome FASTA path or URL</x:v>
+      </x:c>
+      <x:c r="C32" s="68"/>
+      <x:c r="D32" s="20" t="str">
+        <x:v>Optional custom reference set. With STAR, provide genome and GTF. With Salmon genomic decoys, also provide transcripts.</x:v>
+      </x:c>
+      <x:c r="E32" s="39" t="str">
+        <x:v>reference_genome</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="51" customHeight="1">
+      <x:c r="A33" s="66" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B33" s="66" t="str">
+        <x:v>Custom transcriptome FASTA path or URL</x:v>
+      </x:c>
+      <x:c r="C33" s="68"/>
+      <x:c r="D33" s="20" t="str">
+        <x:v>Salmon custom reference requires transcripts and GTF; genomic decoys additionally need genome. IDs must match annotation.</x:v>
+      </x:c>
+      <x:c r="E33" s="39" t="str">
+        <x:v>reference_transcriptome</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="51" customHeight="1">
+      <x:c r="A34" s="66" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B34" s="66" t="str">
+        <x:v>Custom annotation GTF path or URL</x:v>
+      </x:c>
+      <x:c r="C34" s="68"/>
+      <x:c r="D34" s="20" t="str">
+        <x:v>Use the matching assembly/release. If any custom reference is supplied, provide the complete required set.</x:v>
+      </x:c>
+      <x:c r="E34" s="39" t="str">
+        <x:v>reference_gtf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="51" customHeight="1">
+      <x:c r="A35" s="66" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B35" s="66" t="str">
+        <x:v>Salmon decoy profile</x:v>
+      </x:c>
+      <x:c r="C35" s="68" t="str">
+        <x:v>genome</x:v>
+      </x:c>
+      <x:c r="D35" s="20" t="str">
+        <x:v>genome is the new-project default. transcriptome only explicitly disables decoys. STAR does not use this setting.</x:v>
+      </x:c>
+      <x:c r="E35" s="39" t="str">
+        <x:v>reference_decoys</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="51" customHeight="1">
+      <x:c r="A36" s="66" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B36" s="66" t="str">
+        <x:v>Poly-G trimming</x:v>
+      </x:c>
+      <x:c r="C36" s="68" t="str">
+        <x:v>auto</x:v>
+      </x:c>
+      <x:c r="D36" s="20" t="str">
+        <x:v>auto uses fastp instrument-header detection. Choose on or off when the library protocol requires it.</x:v>
+      </x:c>
+      <x:c r="E36" s="39" t="str">
+        <x:v>preprocess_poly_g</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="51" customHeight="1">
+      <x:c r="A37" s="66" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B37" s="66" t="str">
+        <x:v>Explicit R1 adapter sequence</x:v>
+      </x:c>
+      <x:c r="C37" s="68"/>
+      <x:c r="D37" s="20" t="str">
+        <x:v>Optional A/C/G/T sequence. Blank uses the bulk processor auto-detection. Kit-specific processing is not implied.</x:v>
+      </x:c>
+      <x:c r="E37" s="39" t="str">
+        <x:v>preprocess_adapter_r1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="51" customHeight="1">
+      <x:c r="A38" s="66" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B38" s="66" t="str">
+        <x:v>Explicit R2 adapter sequence</x:v>
+      </x:c>
+      <x:c r="C38" s="68"/>
+      <x:c r="D38" s="20" t="str">
+        <x:v>Paired reads only; also supply R1 adapter. Blank uses the R1 sequence when R1 is explicit.</x:v>
+      </x:c>
+      <x:c r="E38" s="39" t="str">
+        <x:v>preprocess_adapter_r2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="51" customHeight="1">
+      <x:c r="A39" s="66" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B39" s="66" t="str">
+        <x:v>Minimum retained read length (nt)</x:v>
+      </x:c>
+      <x:c r="C39" s="69" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D39" s="20" t="str">
+        <x:v>Bulk minimum after processing. This is not a small-RNA size-selection profile.</x:v>
+      </x:c>
+      <x:c r="E39" s="39" t="str">
+        <x:v>preprocess_minimum_length</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
     <x:mergeCell ref="A2:D2"/>
   </x:mergeCells>
-  <x:dataValidations count="15">
+  <x:dataValidations count="20">
     <x:dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C10">
       <x:formula1>"NovaSeq,NextSeq,MiSeq,Other Illumina,don't know"</x:formula1>
     </x:dataValidation>
@@ -1285,6 +1474,22 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C28">
       <x:formula1>"no,yes,don't know"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C30">
+      <x:formula1>"auto,salmon,star"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C31">
+      <x:formula1>"auto,limma_voom,edger_ql,deseq2"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C35">
+      <x:formula1>"genome,transcriptome only"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C36">
+      <x:formula1>"auto,on,off"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="C39">
+      <x:formula1>1</x:formula1>
+      <x:formula2>10000</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>